<commit_message>
Signup tracker: USCIS developer team agl_developersupport created; next steps recorded
</commit_message>
<xml_diff>
--- a/store/vendors/AGL_Vendor_Signup_Playbook.xlsx
+++ b/store/vendors/AGL_Vendor_Signup_Playbook.xlsx
@@ -6169,7 +6169,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Founder's developer.uscis.gov account (exists) → register an app → request Case Status API access</t>
+          <t>Founder's developer.uscis.gov team 'agl_developersupport' (created 2026-10-14) → register an app under the team → request Case Status API access</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>Spec: ai-office/projects/real-apps/specs/Uscis-Case-v2.md. The portal username stays in the founder vault, not in this file.</t>
+          <t>Team agl_developersupport exists (founder, 2026-10-14; page requires sign-in — HTTP 403 to an anonymous check). Next: register the Uscis-Case app under the team, request Case Status (and FOIA, if listed) API access, then put the sandbox client ID/secret into Supabase Edge Function secrets. Spec: ai-office/projects/real-apps/specs/Uscis-Case-v2.md. Portal username stays in the founder vault.</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Signup tracker: USCIS app approved (Case Status + first-case sandboxes); keys must be rotated before use (exposed in chat) — no key material recorded
</commit_message>
<xml_diff>
--- a/store/vendors/AGL_Vendor_Signup_Playbook.xlsx
+++ b/store/vendors/AGL_Vendor_Signup_Playbook.xlsx
@@ -6218,7 +6218,7 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>Team agl_developersupport exists (founder, 2026-10-14; page requires sign-in — HTTP 403 to an anonymous check). Next: register the Uscis-Case app under the team, request Case Status (and FOIA, if listed) API access, then put the sandbox client ID/secret into Supabase Edge Function secrets. Spec: ai-office/projects/real-apps/specs/Uscis-Case-v2.md. Portal username stays in the founder vault.</t>
+          <t>Team agl_developersupport: Uscis-Case app APPROVED; products enabled: 'Case Status API - Sandbox' and 'first-case-sbox' (likely the FIRST/FOIA sandbox — verify); 2 keys issued 2026-07-01, sandbox only — production access not yet requested/granted. 2026-10-14: both client secrets were pasted into a chat — ROTATE them in the portal before use. Store the new values only as Supabase Edge Function secrets (USCIS_CLIENT_ID / USCIS_CLIENT_SECRET); never in chat or git. Spec: ai-office/projects/real-apps/specs/Uscis-Case-v2.md.</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
@@ -6233,9 +6233,9 @@
       <c r="W48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>P4</t>
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -6245,63 +6245,63 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>OpenAI API</t>
+          <t>USCIS FOIA</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Official USCIS FOIA portal; check developer.uscis.gov for a FOIA API</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>https://platform.openai.com/signup</t>
+          <t>https://first.uscis.gov/</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>HTTP 403 to automated check — open in a browser</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Verify on developer.uscis.gov</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Verify</t>
         </is>
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>Dashboard → API keys → Create</t>
+          <t>If an API exists: developer portal app credentials; otherwise none (user files on the official portal)</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret if an API exists</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr"/>
-      <c r="L49" s="7" t="inlineStr">
-        <is>
-          <t>Photriya; HerJourney; daily-pulse</t>
-        </is>
-      </c>
+      <c r="L49" s="7" t="inlineStr"/>
       <c r="M49" s="7" t="inlineStr"/>
       <c r="N49" s="7" t="inlineStr"/>
       <c r="O49" s="7" t="inlineStr">
         <is>
-          <t>Usage-based</t>
+          <t>Verify</t>
         </is>
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="Q49" s="7" t="inlineStr"/>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="Q49" s="7" t="inlineStr">
+        <is>
+          <t>The team's app has 'first-case-sbox' enabled (2026-10-14) — likely the FIRST (FOIA) sandbox API; verify its endpoints on developer.uscis.gov.</t>
+        </is>
+      </c>
       <c r="R49" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -6314,19 +6314,19 @@
       <c r="W49" s="7" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>P4</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>6 Optional monitoring</t>
+          <t>5 AI / server-side keys</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Sentry</t>
+          <t>OpenAI API</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -6336,12 +6336,12 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>https://sentry.io/signup/</t>
+          <t>https://platform.openai.com/signup</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>HTTP 403 to automated check — open in a browser</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -6351,38 +6351,30 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>DSN</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>Project → Settings → Client Keys (DSN)</t>
+          <t>Dashboard → API keys → Create</t>
         </is>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>SENTRY_DSN define (DriftDate, NexusTransferPay)</t>
-        </is>
-      </c>
-      <c r="K50" s="7" t="inlineStr">
-        <is>
-          <t>DriftDate; NexusTransferPay</t>
-        </is>
-      </c>
-      <c r="L50" s="7" t="inlineStr"/>
-      <c r="M50" s="7" t="inlineStr">
-        <is>
-          <t>SENTRY_DSN</t>
-        </is>
-      </c>
-      <c r="N50" s="7" t="inlineStr">
-        <is>
-          <t>DriftDate: SENTRY_DSN: EMPTY in release | NexusTransferPay: SENTRY_DSN: EMPTY in release</t>
-        </is>
-      </c>
+          <t>Supabase Edge Function secret — never in the app</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr"/>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>Photriya; HerJourney; daily-pulse</t>
+        </is>
+      </c>
+      <c r="M50" s="7" t="inlineStr"/>
+      <c r="N50" s="7" t="inlineStr"/>
       <c r="O50" s="7" t="inlineStr">
         <is>
-          <t>Free tier</t>
+          <t>Usage-based</t>
         </is>
       </c>
       <c r="P50" s="7" t="inlineStr">
@@ -6390,11 +6382,7 @@
           <t>Instant</t>
         </is>
       </c>
-      <c r="Q50" s="7" t="inlineStr">
-        <is>
-          <t>Optional — Crashlytics already covers crashes</t>
-        </is>
-      </c>
+      <c r="Q50" s="7" t="inlineStr"/>
       <c r="R50" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -6407,9 +6395,9 @@
       <c r="W50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>P4</t>
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -6419,7 +6407,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>PostHog</t>
+          <t>Sentry</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -6429,7 +6417,7 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>https://us.posthog.com/signup</t>
+          <t>https://sentry.io/signup/</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
@@ -6444,27 +6432,35 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>Project key</t>
+          <t>DSN</t>
         </is>
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Project settings → Project API key</t>
+          <t>Project → Settings → Client Keys (DSN)</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>POSTHOG_API_KEY (MyHealth)</t>
-        </is>
-      </c>
-      <c r="K51" s="7" t="inlineStr"/>
-      <c r="L51" s="7" t="inlineStr">
-        <is>
-          <t>MyHealth</t>
-        </is>
-      </c>
-      <c r="M51" s="7" t="inlineStr"/>
-      <c r="N51" s="7" t="inlineStr"/>
+          <t>SENTRY_DSN define (DriftDate, NexusTransferPay)</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>DriftDate; NexusTransferPay</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr"/>
+      <c r="M51" s="7" t="inlineStr">
+        <is>
+          <t>SENTRY_DSN</t>
+        </is>
+      </c>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>DriftDate: SENTRY_DSN: EMPTY in release | NexusTransferPay: SENTRY_DSN: EMPTY in release</t>
+        </is>
+      </c>
       <c r="O51" s="7" t="inlineStr">
         <is>
           <t>Free tier</t>
@@ -6477,7 +6473,7 @@
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Optional — Crashlytics already covers crashes</t>
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr">
@@ -6499,22 +6495,22 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>7 Later (no app uses it yet)</t>
+          <t>6 Optional monitoring</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>ADS-B Exchange</t>
+          <t>PostHog</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>https://www.adsbexchange.com/</t>
+          <t>https://us.posthog.com/signup</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -6529,30 +6525,30 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Project key</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>Project settings → Project API key</t>
         </is>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>POSTHOG_API_KEY (MyHealth)</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr"/>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute; AeroSwift</t>
+          <t>MyHealth</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr"/>
       <c r="N52" s="7" t="inlineStr"/>
       <c r="O52" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Free tier</t>
         </is>
       </c>
       <c r="P52" s="7" t="inlineStr">
@@ -6562,7 +6558,7 @@
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>Signing up earns nothing until an app is built to use it</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
@@ -6589,17 +6585,17 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Agoda Partner Hub</t>
+          <t>ADS-B Exchange</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>https://partners.agoda.com/</t>
+          <t>https://www.adsbexchange.com/</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -6609,40 +6605,40 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr"/>
       <c r="L53" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>PilotEnRoute; AeroSwift</t>
         </is>
       </c>
       <c r="M53" s="7" t="inlineStr"/>
       <c r="N53" s="7" t="inlineStr"/>
       <c r="O53" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q53" s="7" t="inlineStr">
@@ -6674,7 +6670,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Airalo</t>
+          <t>Agoda Partner Hub</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -6684,7 +6680,7 @@
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>https://partners.airalo.com/</t>
+          <t>https://partners.agoda.com/</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -6759,60 +6755,60 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Airplanes.Live</t>
+          <t>Airalo</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>https://airplanes.live/</t>
+          <t>https://partners.airalo.com/</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Exists — bot-protected (Cloudflare check); open in a browser</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K55" s="7" t="inlineStr"/>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>AeroSwift; PilotEnRoute</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M55" s="7" t="inlineStr"/>
       <c r="N55" s="7" t="inlineStr"/>
       <c r="O55" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q55" s="7" t="inlineStr">
@@ -6844,17 +6840,17 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Allianz Partners</t>
+          <t>Airplanes.Live</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>https://www.allianz-partners.com/</t>
+          <t>https://airplanes.live/</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
@@ -6864,40 +6860,40 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr"/>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>AeroSwift; PilotEnRoute</t>
         </is>
       </c>
       <c r="M56" s="7" t="inlineStr"/>
       <c r="N56" s="7" t="inlineStr"/>
       <c r="O56" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q56" s="7" t="inlineStr">
@@ -6929,60 +6925,60 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Alpha Vantage</t>
+          <t>Allianz Partners</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>https://www.alphavantage.co/support/#api-key</t>
+          <t>https://www.allianz-partners.com/</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>Exists — bot-protected (Cloudflare check); open in a browser</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr"/>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>ApexMarketWatch; daily-pulse</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M57" s="7" t="inlineStr"/>
       <c r="N57" s="7" t="inlineStr"/>
       <c r="O57" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P57" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q57" s="7" t="inlineStr">
@@ -7014,7 +7010,7 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Amadeus for Developers</t>
+          <t>Alpha Vantage</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -7024,12 +7020,12 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>https://developers.amadeus.com/register</t>
+          <t>https://www.alphavantage.co/support/#api-key</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200), lands on https://developers.amadeus.com/</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -7055,7 +7051,7 @@
       <c r="K58" s="7" t="inlineStr"/>
       <c r="L58" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>ApexMarketWatch; daily-pulse</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr"/>
@@ -7099,7 +7095,7 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Auth0</t>
+          <t>Amadeus for Developers</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -7109,12 +7105,12 @@
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>https://auth0.com/signup</t>
+          <t>https://developers.amadeus.com/register</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>OK (HTTP 200), lands on https://developers.amadeus.com/</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -7138,7 +7134,11 @@
         </is>
       </c>
       <c r="K59" s="7" t="inlineStr"/>
-      <c r="L59" s="7" t="inlineStr"/>
+      <c r="L59" s="7" t="inlineStr">
+        <is>
+          <t>TripNest</t>
+        </is>
+      </c>
       <c r="M59" s="7" t="inlineStr"/>
       <c r="N59" s="7" t="inlineStr"/>
       <c r="O59" s="7" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Aviationstack</t>
+          <t>Auth0</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>https://aviationstack.com/signup/free</t>
+          <t>https://auth0.com/signup</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
@@ -7219,11 +7219,7 @@
         </is>
       </c>
       <c r="K60" s="7" t="inlineStr"/>
-      <c r="L60" s="7" t="inlineStr">
-        <is>
-          <t>AeroSwift; PilotEnRoute</t>
-        </is>
-      </c>
+      <c r="L60" s="7" t="inlineStr"/>
       <c r="M60" s="7" t="inlineStr"/>
       <c r="N60" s="7" t="inlineStr"/>
       <c r="O60" s="7" t="inlineStr">
@@ -7265,17 +7261,17 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Bounce</t>
+          <t>Aviationstack</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>https://bounce.com/</t>
+          <t>https://aviationstack.com/signup/free</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
@@ -7285,40 +7281,40 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K61" s="7" t="inlineStr"/>
       <c r="L61" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>AeroSwift; PilotEnRoute</t>
         </is>
       </c>
       <c r="M61" s="7" t="inlineStr"/>
       <c r="N61" s="7" t="inlineStr"/>
       <c r="O61" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q61" s="7" t="inlineStr">
@@ -7350,42 +7346,42 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>CarTrawler</t>
+          <t>Bounce</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>https://www.cartrawler.com/</t>
+          <t>https://bounce.com/</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200), lands on https://corporate.cartrawler.com/en-gb/</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr"/>
@@ -7398,12 +7394,12 @@
       <c r="N62" s="7" t="inlineStr"/>
       <c r="O62" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P62" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q62" s="7" t="inlineStr">
@@ -7435,60 +7431,60 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>CheckWX</t>
+          <t>CarTrawler</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>https://www.checkwxapi.com/</t>
+          <t>https://www.cartrawler.com/</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>OK (HTTP 200), lands on https://corporate.cartrawler.com/en-gb/</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr"/>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M63" s="7" t="inlineStr"/>
       <c r="N63" s="7" t="inlineStr"/>
       <c r="O63" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q63" s="7" t="inlineStr">
@@ -7520,17 +7516,17 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Cirium</t>
+          <t>CheckWX</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>https://www.cirium.com/</t>
+          <t>https://www.checkwxapi.com/</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
@@ -7540,40 +7536,40 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr"/>
       <c r="L64" s="7" t="inlineStr">
         <is>
-          <t>AeroSwift; PilotEnRoute</t>
+          <t>PilotEnRoute</t>
         </is>
       </c>
       <c r="M64" s="7" t="inlineStr"/>
       <c r="N64" s="7" t="inlineStr"/>
       <c r="O64" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P64" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q64" s="7" t="inlineStr">
@@ -7605,7 +7601,7 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Cover Genius</t>
+          <t>Cirium</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -7615,7 +7611,7 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>https://covergenius.com/</t>
+          <t>https://www.cirium.com/</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
@@ -7646,7 +7642,7 @@
       <c r="K65" s="7" t="inlineStr"/>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>AeroSwift; PilotEnRoute</t>
         </is>
       </c>
       <c r="M65" s="7" t="inlineStr"/>
@@ -7690,17 +7686,17 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>DiscoverCars</t>
+          <t>Cover Genius</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>https://www.discovercars.com/affiliate</t>
+          <t>https://covergenius.com/</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
@@ -7710,22 +7706,22 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr"/>
@@ -7738,12 +7734,12 @@
       <c r="N66" s="7" t="inlineStr"/>
       <c r="O66" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q66" s="7" t="inlineStr">
@@ -7775,17 +7771,17 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Distribusion</t>
+          <t>DiscoverCars</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>https://www.distribusion.com/</t>
+          <t>https://www.discovercars.com/affiliate</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
@@ -7795,22 +7791,22 @@
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K67" s="7" t="inlineStr"/>
@@ -7823,12 +7819,12 @@
       <c r="N67" s="7" t="inlineStr"/>
       <c r="O67" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q67" s="7" t="inlineStr">
@@ -7860,7 +7856,7 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Dragonpass</t>
+          <t>Distribusion</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -7870,7 +7866,7 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>https://www.dragonpass.com/</t>
+          <t>https://www.distribusion.com/</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr">
@@ -7945,17 +7941,17 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Duffel</t>
+          <t>Dragonpass</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>https://app.duffel.com/join</t>
+          <t>https://www.dragonpass.com/</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -7965,22 +7961,22 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K69" s="7" t="inlineStr"/>
@@ -7993,12 +7989,12 @@
       <c r="N69" s="7" t="inlineStr"/>
       <c r="O69" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P69" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q69" s="7" t="inlineStr">
@@ -8030,7 +8026,7 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Edamam</t>
+          <t>Duffel</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -8040,7 +8036,7 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>https://developer.edamam.com/</t>
+          <t>https://app.duffel.com/join</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr">
@@ -8071,7 +8067,7 @@
       <c r="K70" s="7" t="inlineStr"/>
       <c r="L70" s="7" t="inlineStr">
         <is>
-          <t>ChefCount; GroceryMatch</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M70" s="7" t="inlineStr"/>
@@ -8115,7 +8111,7 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Finnhub</t>
+          <t>Edamam</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -8125,7 +8121,7 @@
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>https://finnhub.io/</t>
+          <t>https://developer.edamam.com/</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -8156,7 +8152,7 @@
       <c r="K71" s="7" t="inlineStr"/>
       <c r="L71" s="7" t="inlineStr">
         <is>
-          <t>ApexMarketWatch; daily-pulse</t>
+          <t>ChefCount; GroceryMatch</t>
         </is>
       </c>
       <c r="M71" s="7" t="inlineStr"/>
@@ -8200,7 +8196,7 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>FlightAware AeroAPI</t>
+          <t>Finnhub</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -8210,7 +8206,7 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>https://www.flightaware.com/aeroapi/portal</t>
+          <t>https://finnhub.io/</t>
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr">
@@ -8241,7 +8237,7 @@
       <c r="K72" s="7" t="inlineStr"/>
       <c r="L72" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute; AeroSwift</t>
+          <t>ApexMarketWatch; daily-pulse</t>
         </is>
       </c>
       <c r="M72" s="7" t="inlineStr"/>
@@ -8285,17 +8281,17 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>ForeFlight</t>
+          <t>FlightAware AeroAPI</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>https://foreflight.com/</t>
+          <t>https://www.flightaware.com/aeroapi/portal</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
@@ -8305,40 +8301,40 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr"/>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute</t>
+          <t>PilotEnRoute; AeroSwift</t>
         </is>
       </c>
       <c r="M73" s="7" t="inlineStr"/>
       <c r="N73" s="7" t="inlineStr"/>
       <c r="O73" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P73" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q73" s="7" t="inlineStr">
@@ -8370,7 +8366,7 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>Garmin Aviation</t>
+          <t>ForeFlight</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -8380,7 +8376,7 @@
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>https://www.garmin.com/en-US/c/aviation/</t>
+          <t>https://foreflight.com/</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr">
@@ -8455,17 +8451,17 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>GetYourGuide</t>
+          <t>Garmin Aviation</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>https://partner.getyourguide.com/</t>
+          <t>https://www.garmin.com/en-US/c/aviation/</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
@@ -8475,40 +8471,40 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K75" s="7" t="inlineStr"/>
       <c r="L75" s="7" t="inlineStr">
         <is>
-          <t>TripNest; EventSpark</t>
+          <t>PilotEnRoute</t>
         </is>
       </c>
       <c r="M75" s="7" t="inlineStr"/>
       <c r="N75" s="7" t="inlineStr"/>
       <c r="O75" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P75" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q75" s="7" t="inlineStr">
@@ -8540,17 +8536,17 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>GNews</t>
+          <t>GetYourGuide</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>https://gnews.io/</t>
+          <t>https://partner.getyourguide.com/</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
@@ -8560,40 +8556,40 @@
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I76" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J76" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K76" s="7" t="inlineStr"/>
       <c r="L76" s="7" t="inlineStr">
         <is>
-          <t>daily-pulse; NewsBoard</t>
+          <t>TripNest; EventSpark</t>
         </is>
       </c>
       <c r="M76" s="7" t="inlineStr"/>
       <c r="N76" s="7" t="inlineStr"/>
       <c r="O76" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P76" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q76" s="7" t="inlineStr">
@@ -8625,17 +8621,17 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Holafly</t>
+          <t>GNews</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>https://esim.holafly.com/</t>
+          <t>https://gnews.io/</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr">
@@ -8645,40 +8641,40 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J77" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K77" s="7" t="inlineStr"/>
       <c r="L77" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>daily-pulse; NewsBoard</t>
         </is>
       </c>
       <c r="M77" s="7" t="inlineStr"/>
       <c r="N77" s="7" t="inlineStr"/>
       <c r="O77" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P77" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q77" s="7" t="inlineStr">
@@ -8710,7 +8706,7 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>HomeToGo</t>
+          <t>Holafly</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -8720,7 +8716,7 @@
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>https://www.hometogo.com/</t>
+          <t>https://esim.holafly.com/</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
@@ -8795,17 +8791,17 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Hotelbeds</t>
+          <t>HomeToGo</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>https://developer.hotelbeds.com/</t>
+          <t>https://www.hometogo.com/</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
@@ -8815,22 +8811,22 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K79" s="7" t="inlineStr"/>
@@ -8843,12 +8839,12 @@
       <c r="N79" s="7" t="inlineStr"/>
       <c r="O79" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P79" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q79" s="7" t="inlineStr">
@@ -8880,17 +8876,17 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Jayride</t>
+          <t>Hotelbeds</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>https://www.jayride.com/</t>
+          <t>https://developer.hotelbeds.com/</t>
         </is>
       </c>
       <c r="F80" s="7" t="inlineStr">
@@ -8900,22 +8896,22 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J80" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K80" s="7" t="inlineStr"/>
@@ -8928,12 +8924,12 @@
       <c r="N80" s="7" t="inlineStr"/>
       <c r="O80" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P80" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q80" s="7" t="inlineStr">
@@ -8965,17 +8961,17 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Kiwi.com Tequila</t>
+          <t>Jayride</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>https://tequila.kiwi.com/</t>
+          <t>https://www.jayride.com/</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr">
@@ -8985,22 +8981,22 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J81" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K81" s="7" t="inlineStr"/>
@@ -9013,12 +9009,12 @@
       <c r="N81" s="7" t="inlineStr"/>
       <c r="O81" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P81" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q81" s="7" t="inlineStr">
@@ -9050,7 +9046,7 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>LoungeKey</t>
+          <t>Kiwi.com Tequila</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
@@ -9060,7 +9056,7 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>https://www.loungekey.com/</t>
+          <t>https://tequila.kiwi.com/</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr">
@@ -9135,17 +9131,17 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Mapbox</t>
+          <t>LoungeKey</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>https://account.mapbox.com/auth/signup/</t>
+          <t>https://www.loungekey.com/</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
@@ -9155,40 +9151,40 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J83" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K83" s="7" t="inlineStr"/>
       <c r="L83" s="7" t="inlineStr">
         <is>
-          <t>NearServe; iMaps</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M83" s="7" t="inlineStr"/>
       <c r="N83" s="7" t="inlineStr"/>
       <c r="O83" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P83" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q83" s="7" t="inlineStr">
@@ -9220,7 +9216,7 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>NewsAPI</t>
+          <t>Mapbox</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
@@ -9230,7 +9226,7 @@
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>https://newsapi.org/register</t>
+          <t>https://account.mapbox.com/auth/signup/</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr">
@@ -9261,7 +9257,7 @@
       <c r="K84" s="7" t="inlineStr"/>
       <c r="L84" s="7" t="inlineStr">
         <is>
-          <t>daily-pulse; NewsBoard</t>
+          <t>NearServe; iMaps</t>
         </is>
       </c>
       <c r="M84" s="7" t="inlineStr"/>
@@ -9305,60 +9301,60 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Omio</t>
+          <t>NewsAPI</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>https://www.omio.com/</t>
+          <t>https://newsapi.org/register</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>Exists — bot-protected (Cloudflare check); open in a browser</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J85" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K85" s="7" t="inlineStr"/>
       <c r="L85" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>daily-pulse; NewsBoard</t>
         </is>
       </c>
       <c r="M85" s="7" t="inlineStr"/>
       <c r="N85" s="7" t="inlineStr"/>
       <c r="O85" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P85" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q85" s="7" t="inlineStr">
@@ -9390,60 +9386,60 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>OpenAIP</t>
+          <t>Omio</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>https://www.openaip.net/</t>
+          <t>https://www.omio.com/</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>Exists — bot-protected (Cloudflare check); open in a browser</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I86" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J86" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K86" s="7" t="inlineStr"/>
       <c r="L86" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M86" s="7" t="inlineStr"/>
       <c r="N86" s="7" t="inlineStr"/>
       <c r="O86" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P86" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q86" s="7" t="inlineStr">
@@ -9475,7 +9471,7 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>OpenWeather</t>
+          <t>OpenAIP</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
@@ -9485,7 +9481,7 @@
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>https://home.openweathermap.org/users/sign_up</t>
+          <t>https://www.openaip.net/</t>
         </is>
       </c>
       <c r="F87" s="7" t="inlineStr">
@@ -9516,7 +9512,7 @@
       <c r="K87" s="7" t="inlineStr"/>
       <c r="L87" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute; daily-pulse</t>
+          <t>PilotEnRoute</t>
         </is>
       </c>
       <c r="M87" s="7" t="inlineStr"/>
@@ -9560,7 +9556,7 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>Polygon.io</t>
+          <t>OpenWeather</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
@@ -9570,7 +9566,7 @@
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>https://massive.com/dashboard/signup</t>
+          <t>https://home.openweathermap.org/users/sign_up</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr">
@@ -9601,7 +9597,7 @@
       <c r="K88" s="7" t="inlineStr"/>
       <c r="L88" s="7" t="inlineStr">
         <is>
-          <t>ApexMarketWatch; daily-pulse</t>
+          <t>PilotEnRoute; daily-pulse</t>
         </is>
       </c>
       <c r="M88" s="7" t="inlineStr"/>
@@ -9618,7 +9614,7 @@
       </c>
       <c r="Q88" s="7" t="inlineStr">
         <is>
-          <t>Polygon.io now redirects to massive.com (rebranded). Signing up earns nothing until an app is built to use it</t>
+          <t>Signing up earns nothing until an app is built to use it</t>
         </is>
       </c>
       <c r="R88" s="7" t="inlineStr">
@@ -9645,17 +9641,17 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Radical Storage</t>
+          <t>Polygon.io</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Affiliate / partner programme</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>https://radicalstorage.com/</t>
+          <t>https://massive.com/dashboard/signup</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
@@ -9665,45 +9661,45 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>Partner/affiliate ID</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
-          <t>Partner dashboard → your partner/affiliate ID</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J89" s="7" t="inlineStr">
         <is>
-          <t>Build define (public id)</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K89" s="7" t="inlineStr"/>
       <c r="L89" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>ApexMarketWatch; daily-pulse</t>
         </is>
       </c>
       <c r="M89" s="7" t="inlineStr"/>
       <c r="N89" s="7" t="inlineStr"/>
       <c r="O89" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P89" s="7" t="inlineStr">
         <is>
-          <t>Programme review</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q89" s="7" t="inlineStr">
         <is>
-          <t>Signing up earns nothing until an app is built to use it</t>
+          <t>Polygon.io now redirects to massive.com (rebranded). Signing up earns nothing until an app is built to use it</t>
         </is>
       </c>
       <c r="R89" s="7" t="inlineStr">
@@ -9730,17 +9726,17 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>Resend</t>
+          <t>Radical Storage</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Affiliate / partner programme</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>https://resend.com/signup</t>
+          <t>https://radicalstorage.com/</t>
         </is>
       </c>
       <c r="F90" s="7" t="inlineStr">
@@ -9750,36 +9746,40 @@
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company: American Group LLC (legal name, address, EIN), contact email, website https://www.americangroup.ai, the store listing URL of each app that will carry the links, how you promote (in-app links in those apps), estimated monthly users/clicks, payout method (bank/PayPal) and US tax form W-9</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Partner/affiliate ID</t>
         </is>
       </c>
       <c r="I90" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>Partner dashboard → your partner/affiliate ID</t>
         </is>
       </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Build define (public id)</t>
         </is>
       </c>
       <c r="K90" s="7" t="inlineStr"/>
-      <c r="L90" s="7" t="inlineStr"/>
+      <c r="L90" s="7" t="inlineStr">
+        <is>
+          <t>TripNest</t>
+        </is>
+      </c>
       <c r="M90" s="7" t="inlineStr"/>
       <c r="N90" s="7" t="inlineStr"/>
       <c r="O90" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="P90" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Programme review</t>
         </is>
       </c>
       <c r="Q90" s="7" t="inlineStr">
@@ -9811,60 +9811,56 @@
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Rome2Rio</t>
+          <t>Resend</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>https://www.rome2rio.com/</t>
+          <t>https://resend.com/signup</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>Exists — bot-protected (Cloudflare check); open in a browser</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J91" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K91" s="7" t="inlineStr"/>
-      <c r="L91" s="7" t="inlineStr">
-        <is>
-          <t>TripNest</t>
-        </is>
-      </c>
+      <c r="L91" s="7" t="inlineStr"/>
       <c r="M91" s="7" t="inlineStr"/>
       <c r="N91" s="7" t="inlineStr"/>
       <c r="O91" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P91" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q91" s="7" t="inlineStr">
@@ -9896,7 +9892,7 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>Sabre</t>
+          <t>Rome2Rio</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
@@ -9906,12 +9902,12 @@
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>https://developer.sabre.com/</t>
+          <t>https://www.rome2rio.com/</t>
         </is>
       </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>Exists — bot-protected (Cloudflare check); open in a browser</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
@@ -9981,56 +9977,60 @@
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>SendGrid</t>
+          <t>Sabre</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>https://signup.sendgrid.com/</t>
+          <t>https://developer.sabre.com/</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200), lands on https://login.sendgrid.com/unified_login/start?screen_hint=signup</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I93" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J93" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K93" s="7" t="inlineStr"/>
-      <c r="L93" s="7" t="inlineStr"/>
+      <c r="L93" s="7" t="inlineStr">
+        <is>
+          <t>TripNest</t>
+        </is>
+      </c>
       <c r="M93" s="7" t="inlineStr"/>
       <c r="N93" s="7" t="inlineStr"/>
       <c r="O93" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P93" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q93" s="7" t="inlineStr">
@@ -10062,60 +10062,56 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>Skyscanner Partners</t>
+          <t>SendGrid</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>https://www.partners.skyscanner.net/</t>
+          <t>https://signup.sendgrid.com/</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>OK (HTTP 200), lands on https://login.sendgrid.com/unified_login/start?screen_hint=signup</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I94" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J94" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K94" s="7" t="inlineStr"/>
-      <c r="L94" s="7" t="inlineStr">
-        <is>
-          <t>TripNest</t>
-        </is>
-      </c>
+      <c r="L94" s="7" t="inlineStr"/>
       <c r="M94" s="7" t="inlineStr"/>
       <c r="N94" s="7" t="inlineStr"/>
       <c r="O94" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P94" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q94" s="7" t="inlineStr">
@@ -10147,17 +10143,17 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Spoonacular</t>
+          <t>Skyscanner Partners</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Direct API account</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>https://spoonacular.com/food-api/console#Dashboard</t>
+          <t>https://www.partners.skyscanner.net/</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
@@ -10167,40 +10163,40 @@
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
-          <t>API key</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
-          <t>Developer dashboard → API keys</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J95" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret — never in the app</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K95" s="7" t="inlineStr"/>
       <c r="L95" s="7" t="inlineStr">
         <is>
-          <t>ChefCount; GroceryMatch</t>
+          <t>TripNest</t>
         </is>
       </c>
       <c r="M95" s="7" t="inlineStr"/>
       <c r="N95" s="7" t="inlineStr"/>
       <c r="O95" s="7" t="inlineStr">
         <is>
-          <t>Free tier / paid plans — confirm on the page</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P95" s="7" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q95" s="7" t="inlineStr">
@@ -10232,7 +10228,7 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Spoonacular</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
@@ -10242,7 +10238,7 @@
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t>https://dashboard.stripe.com/register</t>
+          <t>https://spoonacular.com/food-api/console#Dashboard</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
@@ -10271,7 +10267,11 @@
         </is>
       </c>
       <c r="K96" s="7" t="inlineStr"/>
-      <c r="L96" s="7" t="inlineStr"/>
+      <c r="L96" s="7" t="inlineStr">
+        <is>
+          <t>ChefCount; GroceryMatch</t>
+        </is>
+      </c>
       <c r="M96" s="7" t="inlineStr"/>
       <c r="N96" s="7" t="inlineStr"/>
       <c r="O96" s="7" t="inlineStr">
@@ -10313,7 +10313,7 @@
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>Ticketmaster Discovery API</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -10323,12 +10323,12 @@
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>https://developer-acct.ticketmaster.com/user/register</t>
+          <t>https://dashboard.stripe.com/register</t>
         </is>
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200), lands on https://developer-account.ticketmaster.com/user/login</t>
+          <t>OK (HTTP 200)</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
@@ -10352,11 +10352,7 @@
         </is>
       </c>
       <c r="K97" s="7" t="inlineStr"/>
-      <c r="L97" s="7" t="inlineStr">
-        <is>
-          <t>EventSpark</t>
-        </is>
-      </c>
+      <c r="L97" s="7" t="inlineStr"/>
       <c r="M97" s="7" t="inlineStr"/>
       <c r="N97" s="7" t="inlineStr"/>
       <c r="O97" s="7" t="inlineStr">
@@ -10371,7 +10367,7 @@
       </c>
       <c r="Q97" s="7" t="inlineStr">
         <is>
-          <t>The register URL lands on the developer login page — create the account from there. Signing up earns nothing until an app is built to use it</t>
+          <t>Signing up earns nothing until an app is built to use it</t>
         </is>
       </c>
       <c r="R97" s="7" t="inlineStr">
@@ -10398,7 +10394,7 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>Tomorrow.io</t>
+          <t>Ticketmaster Discovery API</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
@@ -10408,12 +10404,12 @@
       </c>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>https://app.tomorrow.io/signup</t>
+          <t>https://developer-acct.ticketmaster.com/user/register</t>
         </is>
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
-          <t>OK (HTTP 200)</t>
+          <t>OK (HTTP 200), lands on https://developer-account.ticketmaster.com/user/login</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
@@ -10439,7 +10435,7 @@
       <c r="K98" s="7" t="inlineStr"/>
       <c r="L98" s="7" t="inlineStr">
         <is>
-          <t>PilotEnRoute; daily-pulse</t>
+          <t>EventSpark</t>
         </is>
       </c>
       <c r="M98" s="7" t="inlineStr"/>
@@ -10456,7 +10452,7 @@
       </c>
       <c r="Q98" s="7" t="inlineStr">
         <is>
-          <t>Signing up earns nothing until an app is built to use it</t>
+          <t>The register URL lands on the developer login page — create the account from there. Signing up earns nothing until an app is built to use it</t>
         </is>
       </c>
       <c r="R98" s="7" t="inlineStr">
@@ -10483,17 +10479,17 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>Trainline</t>
+          <t>Tomorrow.io</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Commercial partnership</t>
+          <t>Direct API account</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>https://www.thetrainline.com/</t>
+          <t>https://app.tomorrow.io/signup</t>
         </is>
       </c>
       <c r="F99" s="7" t="inlineStr">
@@ -10503,40 +10499,40 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
+          <t>Account email, organisation (American Group LLC), project/app name, intended use; a card for paid tiers</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>Contract + API credentials</t>
+          <t>API key</t>
         </is>
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
-          <t>After contract: credentials from the account manager</t>
+          <t>Developer dashboard → API keys</t>
         </is>
       </c>
       <c r="J99" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret</t>
+          <t>Supabase Edge Function secret — never in the app</t>
         </is>
       </c>
       <c r="K99" s="7" t="inlineStr"/>
       <c r="L99" s="7" t="inlineStr">
         <is>
-          <t>TripNest</t>
+          <t>PilotEnRoute; daily-pulse</t>
         </is>
       </c>
       <c r="M99" s="7" t="inlineStr"/>
       <c r="N99" s="7" t="inlineStr"/>
       <c r="O99" s="7" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Free tier / paid plans — confirm on the page</t>
         </is>
       </c>
       <c r="P99" s="7" t="inlineStr">
         <is>
-          <t>Weeks; sales process</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="Q99" s="7" t="inlineStr">
@@ -10568,7 +10564,7 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>Travelport</t>
+          <t>Trainline</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -10578,7 +10574,7 @@
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t>https://developer.travelport.com/</t>
+          <t>https://www.thetrainline.com/</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr">
@@ -10653,17 +10649,17 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>USCIS FOIA</t>
+          <t>Travelport</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Official USCIS FOIA portal; check developer.uscis.gov for a FOIA API</t>
+          <t>Commercial partnership</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>https://first.uscis.gov/</t>
+          <t>https://developer.travelport.com/</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr">
@@ -10673,41 +10669,45 @@
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>Verify on developer.uscis.gov</t>
+          <t>Company profile, use case, expected search/booking volume, often a sales call and a signed contract before credentials</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Contract + API credentials</t>
         </is>
       </c>
       <c r="I101" s="7" t="inlineStr">
         <is>
-          <t>If an API exists: developer portal app credentials; otherwise none (user files on the official portal)</t>
+          <t>After contract: credentials from the account manager</t>
         </is>
       </c>
       <c r="J101" s="7" t="inlineStr">
         <is>
-          <t>Supabase Edge Function secret if an API exists</t>
+          <t>Supabase Edge Function secret</t>
         </is>
       </c>
       <c r="K101" s="7" t="inlineStr"/>
-      <c r="L101" s="7" t="inlineStr"/>
+      <c r="L101" s="7" t="inlineStr">
+        <is>
+          <t>TripNest</t>
+        </is>
+      </c>
       <c r="M101" s="7" t="inlineStr"/>
       <c r="N101" s="7" t="inlineStr"/>
       <c r="O101" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="P101" s="7" t="inlineStr">
         <is>
-          <t>Verify</t>
+          <t>Weeks; sales process</t>
         </is>
       </c>
       <c r="Q101" s="7" t="inlineStr">
         <is>
-          <t>Uscis-Case v2 FOIA helper</t>
+          <t>Signing up earns nothing until an app is built to use it</t>
         </is>
       </c>
       <c r="R101" s="7" t="inlineStr">
@@ -16401,7 +16401,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Anthropic, RevenueCat, USCIS Developer Portal (Case Status API), OpenAI API</t>
+          <t>Anthropic, RevenueCat, USCIS Developer Portal (Case Status API), USCIS FOIA, OpenAI API</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -16445,7 +16445,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>ADS-B Exchange, Agoda Partner Hub, Airalo, Airplanes.Live, Allianz Partners, Alpha Vantage, Amadeus for Developers, Auth0, Aviationstack, Bounce, CarTrawler, CheckWX, Cirium, Cover Genius, DiscoverCars, Distribusion, Dragonpass, Duffel, Edamam, Finnhub, FlightAware AeroAPI, ForeFlight, Garmin Aviation, GetYourGuide, GNews, Holafly, HomeToGo, Hotelbeds, Jayride, Kiwi.com Tequila, LoungeKey, Mapbox, NewsAPI, Omio, OpenAIP, OpenWeather, Polygon.io, Radical Storage, Resend, Rome2Rio, Sabre, SendGrid, Skyscanner Partners, Spoonacular, Stripe, Ticketmaster Discovery API, Tomorrow.io, Trainline, Travelport, USCIS FOIA, VIPCars, Wanderu, Welcome Pickups</t>
+          <t>ADS-B Exchange, Agoda Partner Hub, Airalo, Airplanes.Live, Allianz Partners, Alpha Vantage, Amadeus for Developers, Auth0, Aviationstack, Bounce, CarTrawler, CheckWX, Cirium, Cover Genius, DiscoverCars, Distribusion, Dragonpass, Duffel, Edamam, Finnhub, FlightAware AeroAPI, ForeFlight, Garmin Aviation, GetYourGuide, GNews, Holafly, HomeToGo, Hotelbeds, Jayride, Kiwi.com Tequila, LoungeKey, Mapbox, NewsAPI, Omio, OpenAIP, OpenWeather, Polygon.io, Radical Storage, Resend, Rome2Rio, Sabre, SendGrid, Skyscanner Partners, Spoonacular, Stripe, Ticketmaster Discovery API, Tomorrow.io, Trainline, Travelport, VIPCars, Wanderu, Welcome Pickups</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Founder decisions for PlantPulse v2; in-place App Store resubmit and Play draft discard scripts; USCIS test reads the snapshot; Sentry tracker row
- specs/PlantPulse-v2.md: founder decision table (2026-10-14)
- scripts/testflight/resolve_and_resubmit.rb: resolve rejected items, resubmit the same submission
- scripts/play_discard_draft.py: delete draft releases on one Play track (refuses non-drafts)
- scripts/uscis_sandbox_test.py: fields live under 'snapshot'; cache hit needs USCIS_STORE=db
- docs/API_ACTIONS.md: rows for the two new scripts
- store/vendors: Sentry org exists (signup_playbook --check: no secret-like values)
</commit_message>
<xml_diff>
--- a/store/vendors/AGL_Vendor_Signup_Playbook.xlsx
+++ b/store/vendors/AGL_Vendor_Signup_Playbook.xlsx
@@ -1863,7 +1863,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PRODUCTION_DRAFT_STAGED</t>
+          <t>INTERNAL_ONLY</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Account exists: Sentry organization 'american-group-llc' (founder, 2026-10-14)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -6473,7 +6473,7 @@
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>Optional — Crashlytics already covers crashes</t>
+          <t>Org american-group-llc exists (sign-in page confirmed 2026-10-14). Only DriftDate uses Sentry today (sentry_flutter + SENTRY_DSN, empty in builds); MyHealth reads SENTRY_DSN without the SDK (dead config); NexusTransferPay no longer uses it. Next: a 'driftdate' Flutter project → DSN (public by design) passed at build time; privacy label adds crash data. Other apps use Crashlytics — no duplicate SDK.</t>
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr">

</xml_diff>